<commit_message>
journal of polymer science
Modified for journal of polymer science submission
</commit_message>
<xml_diff>
--- a/data/XY/data_set_3&4/data_set_3&4_SMILES&objective_function.xlsx
+++ b/data/XY/data_set_3&4/data_set_3&4_SMILES&objective_function.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81806\0_doctor_reserch\1_nitroxide\paper\250604_3rd_submit_M06\github\data\XY\data_set_3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81806\0_doctor_reserch\1_nitroxide\paper\250604_3rd_submit_M06\github\Mechanism_Oriented_Reaction_Descriptors_for_living_radical_polymerization\data\XY\data_set_3&amp;4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7701114B-FFFB-4A48-8A99-A8525EB71192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F5F915-88A2-4FC1-89D7-079403AB971E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-3045" windowWidth="29040" windowHeight="15720" xr2:uid="{8B902C3A-E153-43EA-81AD-E54E79E1E759}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8B902C3A-E153-43EA-81AD-E54E79E1E759}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>number</t>
     <phoneticPr fontId="2"/>
@@ -47,6 +47,92 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
+    <t>[O]N1[C@@](C)(C(OC)=O)CCC[C@]1(C)C(OC)=O</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>[O]N1[C@](C(OC)=O)(C)CCC[C@@]1(C)C(OC)=O</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>[O]N1C(CC)(CC)CC(O)CCC1(CC)CC</t>
+  </si>
+  <si>
+    <t>[O]N1[C@@](CC)(C(OC)=O)CCC[C@]1(C(OC)=O)CC</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>[O]N1[C@@](C)(COC)CCC[C@]1(COC)C</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>[O]N1[C@@](C)(CO[Si](C)(C)C(C)(C)C)CCC[C@]1(CO[Si](C)(C)C(C)(C)C)C</t>
+  </si>
+  <si>
+    <t>CC(C)(C)N([O])C(C1=CC=CC=C1)C(C)C</t>
+  </si>
+  <si>
+    <t>[O]N(C(C)(C)C1)C(C)(C)CC1=O</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>[O]N(C(C)(C)CC1)C(C)(C)CC1=O</t>
+  </si>
+  <si>
+    <t>[O]N(C(C)(C)C1)C(C)(C)CCCC1=O</t>
+  </si>
+  <si>
+    <t>OC1CC(C)(C)N([O])C(C)(C)C1</t>
+  </si>
+  <si>
+    <t>[O]N1C(C)(C)CC(O)CCC1(C)C</t>
+  </si>
+  <si>
+    <t>[O]N1C(C)(C)CCC(O)CCC1(C)C</t>
+  </si>
+  <si>
+    <t>[O]N1C(C)(C)CCCC(O)CC1(C)C</t>
+  </si>
+  <si>
+    <t>O=C1CC(CC)(CC)N([O])C(CC)(CC)C1</t>
+  </si>
+  <si>
+    <t>OC1CC(CC)(CC)N([O])C(CC)(CC)C1</t>
+  </si>
+  <si>
+    <t>O=C1CC(CC)(CC)N([O])C(C)(C)C1</t>
+  </si>
+  <si>
+    <t>[O]N(C(CC)(CC)CC1)C(CC)(CC)CC1=O</t>
+  </si>
+  <si>
+    <t>St_Mn</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>St_PDI</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>St_Conversion</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>nBA_Mn</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>nBA_PDI</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>nBA_Conversion</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>[O]N(C(C)(CC1)C)C(C)(CCC1=O)C</t>
+  </si>
+  <si>
     <t>7 (24)</t>
     <phoneticPr fontId="2"/>
   </si>
@@ -55,94 +141,8 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>[O]N1[C@@](C)(C(OC)=O)CCC[C@]1(C)C(OC)=O</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>[O]N1[C@](C(OC)=O)(C)CCC[C@@]1(C)C(OC)=O</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>[O]N1C(CC)(CC)CC(O)CCC1(CC)CC</t>
-  </si>
-  <si>
-    <t>[O]N1[C@@](CC)(C(OC)=O)CCC[C@]1(C(OC)=O)CC</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>[O]N1[C@@](C)(COC)CCC[C@]1(COC)C</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>[O]N1[C@@](C)(CO[Si](C)(C)C(C)(C)C)CCC[C@]1(CO[Si](C)(C)C(C)(C)C)C</t>
-  </si>
-  <si>
-    <t>CC(C)(C)N([O])C(C1=CC=CC=C1)C(C)C</t>
-  </si>
-  <si>
-    <t>[O]N(C(C)(C)C1)C(C)(C)CC1=O</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>[O]N(C(C)(C)CC1)C(C)(C)CC1=O</t>
-  </si>
-  <si>
-    <t>[O]N(C(C)(C)C1)C(C)(C)CCCC1=O</t>
-  </si>
-  <si>
-    <t>OC1CC(C)(C)N([O])C(C)(C)C1</t>
-  </si>
-  <si>
-    <t>[O]N1C(C)(C)CC(O)CCC1(C)C</t>
-  </si>
-  <si>
-    <t>[O]N1C(C)(C)CCC(O)CCC1(C)C</t>
-  </si>
-  <si>
-    <t>[O]N1C(C)(C)CCCC(O)CC1(C)C</t>
-  </si>
-  <si>
-    <t>O=C1CC(CC)(CC)N([O])C(CC)(CC)C1</t>
-  </si>
-  <si>
-    <t>OC1CC(CC)(CC)N([O])C(CC)(CC)C1</t>
-  </si>
-  <si>
-    <t>O=C1CC(CC)(CC)N([O])C(C)(C)C1</t>
-  </si>
-  <si>
-    <t>[O]N(C(CC)(CC)CC1)C(CC)(CC)CC1=O</t>
-  </si>
-  <si>
-    <t>St_Mn</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>St_PDI</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>St_Conversion</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>13 (28)</t>
     <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>nBA_Mn</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>nBA_PDI</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>nBA_Conversion</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>[O]N(C(C)(CC1)C)C(C)(CCC1=O)C</t>
   </si>
 </sst>
 </file>
@@ -518,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DBB32C-8E6C-48EC-9C73-2F2F715C4DCC}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="4" max="4" width="15.5" bestFit="1" customWidth="1"/>
@@ -530,22 +530,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>2</v>
@@ -565,7 +565,7 @@
         <v>43</v>
       </c>
       <c r="H2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.4">
@@ -582,7 +582,7 @@
         <v>58</v>
       </c>
       <c r="H3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.4">
@@ -599,7 +599,7 @@
         <v>61</v>
       </c>
       <c r="H4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.4">
@@ -616,7 +616,7 @@
         <v>71</v>
       </c>
       <c r="H5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.4">
@@ -633,7 +633,7 @@
         <v>50</v>
       </c>
       <c r="H6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.4">
@@ -650,12 +650,12 @@
         <v>69</v>
       </c>
       <c r="H7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="B8">
         <v>1800</v>
@@ -672,7 +672,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="B9">
         <v>5000</v>
@@ -684,7 +684,7 @@
         <v>51</v>
       </c>
       <c r="H9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.4">
@@ -710,7 +710,7 @@
         <v>13</v>
       </c>
       <c r="H10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.4">
@@ -736,7 +736,7 @@
         <v>59</v>
       </c>
       <c r="H11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.4">
@@ -762,7 +762,7 @@
         <v>71</v>
       </c>
       <c r="H12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.4">
@@ -788,12 +788,12 @@
         <v>55</v>
       </c>
       <c r="H13" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B14">
         <v>2200</v>
@@ -805,7 +805,7 @@
         <v>26</v>
       </c>
       <c r="H14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.4">
@@ -831,7 +831,7 @@
         <v>16</v>
       </c>
       <c r="H15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.4">
@@ -857,7 +857,7 @@
         <v>36</v>
       </c>
       <c r="H16" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.4">
@@ -883,7 +883,7 @@
         <v>17</v>
       </c>
       <c r="H17" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.4">
@@ -900,7 +900,7 @@
         <v>79</v>
       </c>
       <c r="H18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.4">
@@ -917,7 +917,7 @@
         <v>68</v>
       </c>
       <c r="H19" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.4">
@@ -934,7 +934,7 @@
         <v>65</v>
       </c>
       <c r="H20" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.4">
@@ -951,24 +951,7 @@
         <v>66</v>
       </c>
       <c r="H21" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A22" s="1">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>10600</v>
-      </c>
-      <c r="C22">
-        <v>1.64</v>
-      </c>
-      <c r="D22">
-        <v>56</v>
-      </c>
-      <c r="H22" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>